<commit_message>
Actualizar dashboard al corte de agosto 2026
</commit_message>
<xml_diff>
--- a/pagina/data/informe_alcohol_drogas.xlsx
+++ b/pagina/data/informe_alcohol_drogas.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Regiones'!$A$1:$C$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sexo_edad'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Estado_tipo_violencia'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Historico_mensual'!$A$1:$D$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Historico_mensual'!$A$1:$D$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,6 +42,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
@@ -52,9 +55,6 @@
     <font>
       <i val="1"/>
       <color rgb="00595959"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <i val="1"/>
@@ -75,13 +75,19 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin">
@@ -103,22 +109,22 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -501,7 +507,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Centro Emergencia Mujer y Familia · Enero - Julio 2026 (preliminar)</t>
+          <t>Centro Emergencia Mujer y Familia · Enero - Agosto 2026 (preliminar)</t>
         </is>
       </c>
     </row>
@@ -512,7 +518,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>29136</v>
+        <v>33381</v>
       </c>
     </row>
     <row r="5">
@@ -522,7 +528,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>27.9</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +539,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18 10:33</t>
+          <t>2026-09-18 09:54</t>
         </is>
       </c>
     </row>
@@ -584,10 +590,10 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>26898</v>
+        <v>30777</v>
       </c>
       <c r="C2" s="10" t="n">
-        <v>92.3</v>
+        <v>92.2</v>
       </c>
     </row>
     <row r="3">
@@ -597,10 +603,10 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>1197</v>
+        <v>1391</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="4">
@@ -610,7 +616,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>1041</v>
+        <v>1213</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>3.6</v>
@@ -671,7 +677,7 @@
         </is>
       </c>
       <c r="C2" s="9" t="n">
-        <v>28569</v>
+        <v>32735</v>
       </c>
       <c r="D2" s="10" t="n">
         <v>98.09999999999999</v>
@@ -689,7 +695,7 @@
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>567</v>
+        <v>646</v>
       </c>
       <c r="D3" s="10" t="n">
         <v>1.9</v>
@@ -707,7 +713,7 @@
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>28666</v>
+        <v>32857</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>98.40000000000001</v>
@@ -725,7 +731,7 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>470</v>
+        <v>524</v>
       </c>
       <c r="D5" s="10" t="n">
         <v>1.6</v>
@@ -743,10 +749,10 @@
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>17207</v>
+        <v>19773</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>59.1</v>
+        <v>59.2</v>
       </c>
     </row>
     <row r="7">
@@ -761,10 +767,10 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>11929</v>
+        <v>13608</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>40.9</v>
+        <v>40.8</v>
       </c>
     </row>
     <row r="8">
@@ -779,10 +785,10 @@
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>22333</v>
+        <v>25487</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>76.7</v>
+        <v>76.40000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -797,10 +803,10 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>6803</v>
+        <v>7894</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>23.3</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="10">
@@ -815,10 +821,10 @@
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>14470</v>
+        <v>16544</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>49.7</v>
+        <v>49.6</v>
       </c>
     </row>
     <row r="11">
@@ -833,10 +839,10 @@
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>10658</v>
+        <v>12253</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>36.6</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="12">
@@ -851,10 +857,10 @@
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>4008</v>
+        <v>4584</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>13.8</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="13">
@@ -869,10 +875,10 @@
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>16144</v>
+        <v>18459</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>55.4</v>
+        <v>55.3</v>
       </c>
     </row>
     <row r="14">
@@ -887,7 +893,7 @@
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>10549</v>
+        <v>12091</v>
       </c>
       <c r="D14" s="10" t="n">
         <v>36.2</v>
@@ -905,10 +911,10 @@
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>2443</v>
+        <v>2831</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
     </row>
   </sheetData>
@@ -955,10 +961,10 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>4629</v>
+        <v>5290</v>
       </c>
       <c r="C2" s="10" t="n">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="3">
@@ -968,7 +974,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>3165</v>
+        <v>3640</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>10.9</v>
@@ -981,10 +987,10 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>2325</v>
+        <v>2704</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="5">
@@ -994,20 +1000,20 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>1646</v>
+        <v>1847</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>ANCASH</t>
+          <t>LA LIBERTAD</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>1376</v>
+        <v>1570</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>4.7</v>
@@ -1016,11 +1022,11 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>LA LIBERTAD</t>
+          <t>ANCASH</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>1361</v>
+        <v>1565</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>4.7</v>
@@ -1029,27 +1035,27 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>LIMA PROVINCIA</t>
+          <t>AYACUCHO</t>
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>1325</v>
+        <v>1553</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>AYACUCHO</t>
+          <t>LIMA PROVINCIA</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1318</v>
+        <v>1522</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="10">
@@ -1059,7 +1065,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>1236</v>
+        <v>1409</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>4.2</v>
@@ -1072,10 +1078,10 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>1137</v>
+        <v>1247</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="12">
@@ -1085,7 +1091,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>1073</v>
+        <v>1229</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>3.7</v>
@@ -1098,7 +1104,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>921</v>
+        <v>1057</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>3.2</v>
@@ -1111,7 +1117,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>906</v>
+        <v>1030</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>3.1</v>
@@ -1124,20 +1130,20 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>842</v>
+        <v>938</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>TACNA</t>
+          <t>LORETO</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>728</v>
+        <v>833</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>2.5</v>
@@ -1146,14 +1152,14 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>LORETO</t>
+          <t>TACNA</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>709</v>
+        <v>822</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="18">
@@ -1163,7 +1169,7 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>698</v>
+        <v>800</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>2.4</v>
@@ -1176,7 +1182,7 @@
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>638</v>
+        <v>735</v>
       </c>
       <c r="C19" s="10" t="n">
         <v>2.2</v>
@@ -1189,10 +1195,10 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>523</v>
+        <v>630</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="21">
@@ -1202,7 +1208,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>420</v>
+        <v>484</v>
       </c>
       <c r="C21" s="10" t="n">
         <v>1.4</v>
@@ -1215,7 +1221,7 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>418</v>
+        <v>477</v>
       </c>
       <c r="C22" s="10" t="n">
         <v>1.4</v>
@@ -1228,7 +1234,7 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>406</v>
+        <v>468</v>
       </c>
       <c r="C23" s="10" t="n">
         <v>1.4</v>
@@ -1241,7 +1247,7 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>382</v>
+        <v>448</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>1.3</v>
@@ -1254,7 +1260,7 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>352</v>
+        <v>394</v>
       </c>
       <c r="C25" s="10" t="n">
         <v>1.2</v>
@@ -1267,7 +1273,7 @@
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>323</v>
+        <v>363</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>1.1</v>
@@ -1280,7 +1286,7 @@
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>279</v>
+        <v>326</v>
       </c>
       <c r="C27" s="10" t="n">
         <v>1</v>
@@ -1348,19 +1354,19 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C2" s="8" t="n">
-        <v>1396</v>
+        <v>1590</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>1475</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="3">
@@ -1370,19 +1376,19 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>254</v>
+        <v>299</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>25573</v>
+        <v>29302</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>1107</v>
+        <v>1257</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>727</v>
+        <v>841</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>27661</v>
+        <v>31699</v>
       </c>
     </row>
     <row r="4">
@@ -1392,19 +1398,19 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>266</v>
+        <v>314</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>26969</v>
+        <v>30892</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>1148</v>
+        <v>1302</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>753</v>
+        <v>873</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>29136</v>
+        <v>33381</v>
       </c>
     </row>
   </sheetData>
@@ -1469,19 +1475,19 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C2" s="8" t="n">
-        <v>11491</v>
+        <v>13078</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>12427</v>
+        <v>14227</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>2948</v>
+        <v>3438</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>26898</v>
+        <v>30777</v>
       </c>
     </row>
     <row r="3">
@@ -1491,19 +1497,19 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>521</v>
+        <v>611</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>510</v>
+        <v>587</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>162</v>
+        <v>188</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>1197</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="4">
@@ -1516,16 +1522,16 @@
         <v>1</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>443</v>
+        <v>500</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>463</v>
+        <v>556</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>134</v>
+        <v>156</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>1041</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="5">
@@ -1535,19 +1541,19 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>12455</v>
+        <v>14189</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>13400</v>
+        <v>15370</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>3244</v>
+        <v>3782</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>29136</v>
+        <v>33381</v>
       </c>
     </row>
   </sheetData>
@@ -1562,7 +1568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1736,7 +1742,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -1746,17 +1752,17 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>18 a 59 años</t>
+          <t>0 a 17 años</t>
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>3691</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -1770,13 +1776,13 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>3492</v>
+        <v>3691</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -1790,13 +1796,13 @@
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>3746</v>
+        <v>3492</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -1810,13 +1816,13 @@
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>3494</v>
+        <v>3746</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -1830,13 +1836,13 @@
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>3874</v>
+        <v>3494</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -1850,13 +1856,13 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>3636</v>
+        <v>3874</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -1870,13 +1876,13 @@
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>3640</v>
+        <v>3636</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -1886,17 +1892,17 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>60 a más años</t>
+          <t>18 a 59 años</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>155</v>
+        <v>3640</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -1906,17 +1912,17 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>60 a más años</t>
+          <t>18 a 59 años</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>168</v>
+        <v>3729</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -1930,13 +1936,13 @@
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>167</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -1956,7 +1962,7 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -1970,13 +1976,13 @@
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>146</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -1990,13 +1996,13 @@
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>158</v>
+        <v>168</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
@@ -2010,13 +2016,13 @@
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -2026,17 +2032,17 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>60 a más años</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>95</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
@@ -2046,17 +2052,17 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>60 a más años</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>105</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -2066,17 +2072,17 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>60 a más años</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>112</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
@@ -2090,13 +2096,13 @@
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>82</v>
+        <v>95</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -2110,13 +2116,13 @@
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>92</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
@@ -2130,13 +2136,13 @@
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>124</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -2150,93 +2156,93 @@
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>117</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Mujer</t>
+          <t>Hombre</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>0 a 17 años</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>3</v>
+        <v>92</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Mujer</t>
+          <t>Hombre</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>0 a 17 años</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
-        <v>0</v>
+        <v>124</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Mujer</t>
+          <t>Hombre</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>0 a 17 años</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
-        <v>1</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Mujer</t>
+          <t>Hombre</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>0 a 17 años</t>
+          <t>Sin información</t>
         </is>
       </c>
       <c r="D33" s="9" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
@@ -2250,13 +2256,13 @@
         </is>
       </c>
       <c r="D34" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -2270,13 +2276,13 @@
         </is>
       </c>
       <c r="D35" s="9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
@@ -2290,13 +2296,13 @@
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -2306,17 +2312,17 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>18 a 59 años</t>
+          <t>0 a 17 años</t>
         </is>
       </c>
       <c r="D37" s="9" t="n">
-        <v>181</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
@@ -2326,17 +2332,17 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>18 a 59 años</t>
+          <t>0 a 17 años</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>193</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -2346,17 +2352,17 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>18 a 59 años</t>
+          <t>0 a 17 años</t>
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>220</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
@@ -2366,17 +2372,17 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>18 a 59 años</t>
+          <t>0 a 17 años</t>
         </is>
       </c>
       <c r="D40" s="9" t="n">
-        <v>185</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
@@ -2386,17 +2392,17 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>18 a 59 años</t>
+          <t>0 a 17 años</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>170</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
@@ -2410,13 +2416,13 @@
         </is>
       </c>
       <c r="D42" s="9" t="n">
-        <v>228</v>
+        <v>181</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -2430,13 +2436,13 @@
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>219</v>
+        <v>193</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
@@ -2446,17 +2452,17 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>60 a más años</t>
+          <t>18 a 59 años</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>4</v>
+        <v>220</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -2466,17 +2472,17 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>60 a más años</t>
+          <t>18 a 59 años</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>5</v>
+        <v>185</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
@@ -2486,17 +2492,17 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>60 a más años</t>
+          <t>18 a 59 años</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1</v>
+        <v>170</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
@@ -2506,17 +2512,17 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>60 a más años</t>
+          <t>18 a 59 años</t>
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>1</v>
+        <v>228</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
@@ -2526,17 +2532,17 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>60 a más años</t>
+          <t>18 a 59 años</t>
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>15</v>
+        <v>219</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -2546,17 +2552,17 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>60 a más años</t>
+          <t>18 a 59 años</t>
         </is>
       </c>
       <c r="D49" s="9" t="n">
-        <v>9</v>
+        <v>194</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
@@ -2570,13 +2576,13 @@
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -2586,17 +2592,17 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>60 a más años</t>
         </is>
       </c>
       <c r="D51" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
@@ -2606,17 +2612,17 @@
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>60 a más años</t>
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -2626,17 +2632,17 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>60 a más años</t>
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
@@ -2646,17 +2652,17 @@
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>60 a más años</t>
         </is>
       </c>
       <c r="D54" s="9" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -2666,17 +2672,17 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>60 a más años</t>
         </is>
       </c>
       <c r="D55" s="9" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
@@ -2686,35 +2692,195 @@
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Sin información</t>
+          <t>60 a más años</t>
         </is>
       </c>
       <c r="D56" s="9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>60 a más años</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Sin información</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>Sin información</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Sin información</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>Sin información</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>Sin información</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>Sin información</t>
+        </is>
+      </c>
+      <c r="D63" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
           <t>2026-07</t>
         </is>
       </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>Mujer</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
         <is>
           <t>Sin información</t>
         </is>
       </c>
-      <c r="D57" s="9" t="n">
+      <c r="D64" s="9" t="n">
         <v>10</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Mujer</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>Sin información</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D57"/>
+  <autoFilter ref="A1:D65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>